<commit_message>
Fixed dashboard not updating
</commit_message>
<xml_diff>
--- a/claims_analysis_output.xlsx
+++ b/claims_analysis_output.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Open_Aging_Summary" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Open_Tasks_By_Warehouse" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Open_Tasks_Aggregate" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="WH_Please_Respond" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19928,4 +19929,953 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Warehouse (Bucket Name)</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Task ID</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Task Name</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2ikza2RmEUmpvC2y9QXD72UAKY3L</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>JL1Z7000ARM - 04862 - CLEVELAND FORD - S39-01507720 - CLAIM 3042581</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>F9FBrcnLzUuACHCiAb3rsWUAJ5lk</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CHRYSLER MIS-SHIP - SHORT 68465585AC - PO 1318972 - WD5189 - 11.22.25 - CLAIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>FFwFCTxGcUSFlq62I04z-GUAAcql</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>PO 160295-  INV S53513 - JL3Z7000F- QTY 1 -7.1.24</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>JQzX2NGQ00-wn1BaYmR5UWUAAFJq</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CHRYSLER OVERSHIPMENT - PO# 1306422 - PART# 68272789AA - CLAIM 438957</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Z8p-hjf9oUqd8TQpk2SDjmUAMX95</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>PO# 158427 - Q89654 - HL3Z6006D - 1 - 4.22.24 - DENIED 8378358</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>a_CxZwy-n0WX_ksTlIBFDWUAFMdT</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CHRYSLER PICKING ERROR - PO# 1305309 - PART# 68254461AA (short) - Qty 1 - CLAIM 580994 (AD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>iiXW_h4e5ESjrYZQR5eiRWUAK5G6</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ATLANTA - CHRYSLER SHORTAGE - PO 0835616- 68048988AA- SHORT 5  - INV DATE 03/22/2025 - CLAIM  898456 Denied</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>sPJVvzzjdUGlx7aMw_6Ma2UAGBcG</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>PO# 159493 - R62299 - MULTI - 3 - 5.22.24</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>tCcd1QKZsUeL-EanbmjLdWUAEmSi</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>BT4Z7902CRM - 00484 - DUVALL FORD - S39-01483760</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>wJOxBEpChEqCivSUq19h3GUAIbVd</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>GC4Z6007FARM - PO 170983 - 00348 - RIVERSIDE FORD WAREHOUSE - S39-01488276</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>xW034z6DKkO6NjrQDnqPG2UAJOkr</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CHRYSLER SHORTAGE - PO 1304122 - 68053666AB - SHORT 2 - INV DATE 7.27.24 - CLAIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>zv5fVIb2X0-q6PdwUOE3KWUANgrF</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>ATLANTA - CHRYSLER SHORTAGE - PO 316366- PART 53011134AA- SHORT 1  - INV DATE 07/19/2025 - CLAIM 126997 Denied</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Charlotte</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>1SHsEemukUu86AXHSDOeAGUAFQI4</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>DC3Z6007ARM - 08799 - RICHMOND FORD LINCOLN - S39-01412084 - AFS 124199</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Charlotte</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>6XybVE08ok2htYMG2BrXQGUADqdh</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>L1MZ7000G - 00905 - PARKWAY FORD, INC. - IN01559935 - Claim # AFS 127856</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Charlotte</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>8cbssBEZKkSPYzW6DoQcdWUALHce</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>DA5Z7000ARM - 06658 - SANDERS FORD - IN01567831 - 3434166</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Charlotte</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>W3TT7asYFUGKNLhF96FEumUAJX6O</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>K2GZ7000C - P1001365 - 08557 - DOUG HENRY FORD OF AYDEN - IN01564872</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Charlotte</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>YAfUOadp-UeUAAz658g4YGUAImxp</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>CHRYSLER DAMAGE - PO# 1324355 - PART# R8453637AB - 1 - CLAIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Charlotte</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ZCkXOW0C80yTIMhdaCYo92UAKOAE</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>GF1Z6006DRM- 09681- DAVID WILSON FORD - CLAIM 127857</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Flowood</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ObMMFmTpAUu3ku4UBA_AF2UAFQiB</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>CHRYSLER OVERAGE - PO 1301636- PART 68311108AE- OVERAGE 1 - INV DATE - CLAIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>OKC</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Wyy6uN2J0EOYRtzJI6bNpWUAJy1W</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>CHRYSLER SHORTAGE - DUPLICATE TASK IN ERROR MINUS 1 PART - CLOSED TASK!PO 1302893/1302550 - PART # MULTI - SHORT 7 - INV DATE 6.29.24 - CLAIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Ontario</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>6JZfKtg-Q0q8DqfsP4nYlmUAKBAV</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>CHRYSLER DAMAGE - PO 1284768 - R8078840AB - 1 - INV DATE 3.31.23 - CLAIM 883225 (AD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Ontario</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Jl2lZXbSEkq24OwU2YK3FWUAHIlN</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>CHRYSLER DAMAGE PO # 284173 - Part # R2123025AD - CLAIM 886235 (AD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Ontario</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ShQHvZYls02BinKYRX7-i2UAMj_D</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>CHRYSLER WRONG PART - SHORT R8293289AB  - PO 1320798 - CLAIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Ontario</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>UHfMCGoPykK5bJw1klGzVmUAJ1rh</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>FL3Z7902AARM - PO 174471 - 00514 - FORD OF UPLAND - IN01566622</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Ontario</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>VuNjjDXFqU6XsNJr39WejGUAP-Le</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>CHRYSLER DAMAGE - PO# 289919 - PART# R8447797AA - CLAIM 490287</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Ontario</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Xox7001YwEqzihoxH2NRFmUAAGZi</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>CHRYSLER PO#1285577 - PART # R8321378AA - CLAIM 942323 (AD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Ontario</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>YEEEHNOCNU6ibMLX2a0NWWUAJXVw</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>***CHRYSLER PART# R8143186AD QTY.14 - PO 318126 - 332630 - 332643</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Ontario</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>c4ITm8nQ4E2CN4r3GdhI8mUALbwn</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>ONTARIO - CHRYSLER SHORTAGE - PO 0837937- 68346915AA- SHORT 1  - INV DATE 04/05/2025 - CLAIM - 923169 Denied</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Ontario</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>nj3hOH9hZUGhbcC3DfWk1WUAPb84</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>- PO# 61127- INV T45058- PART  JC3Z7000ARM- QTY  1- DATE 08.08.2024 ADDED TO ANOTHER TASK TO FILE CLAIM TOGETHER</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Ontario</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>oKorWTnBMUy3pfF-8nIIjWUANlXO</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>CHRYSLER PICK ERROR  - PART# 68334756AG PO - 1321019 WRONG PART IS 68306203AM - CLAIM 267720</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Ontario</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>u0nBEYulzkOh6WUoKzWB_WUAO_zp</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ONTARIO - CHRYSLER SHORTAGE - PO 0837832- 68315880AA- SHORT 4 - INV DATE 03/29/2025 - CLAIM - 912469 DENIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Ontario</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>uBRoB403c0u0bbdtNcoa_GUAFgyJ</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>***CHRYSLER PICKING ERROR *** PO# 1312348 - PART# 68005435AA - CLAIM 818516 (AD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Ontario</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>woK6YvJvS02ggf-4VNVKsGUADzTt</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>CHRYSLER WRONG PART - PO 1320109 - PART# 68261528AE - QTY 10 - CLAIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Ontario</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>ykU6kfUdr0WzVN_NjqjtEmUAH6d6</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>CHRYSLER WRONG PART - PART# 68515620AA - PO 1320798 - WRONG PART IS 68237096BB 260854</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Ontario</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>zIVaT-mI6Ui7qjqCJq8D42UAF1fU</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>ONTARIO - CHRYSLER SHORTAGE - PO 0823280 - 68477444AA - SHORT 1 - INV DATE 8.24.24 - CLAIM 376318(C), 376329(C), 376337(C), 376344(C), 376352(C), 376355(AD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Orlando</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>C7geTg_mn0q8e2UuED5Fl2UANZ7M</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>PO# 59496 CORRECT PO 160801- INV T15234 - K2GZ7000VRM - QTY 1 - DATE 7.26.24 - 8882613</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Orlando</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>FNB-mfp8g0qJAUYNIpX9rGUAOtph</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>ORLANDO - CHRYSLER PICKING ERROR - PO 1320791 - WRONG PART SHIPPED (R8020952AA-1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Orlando</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>JXQwYM0W3Em8D31SXm_McmUALLYO</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>ORLANDO-CHRYSLER -PO 1318313-68568033AA(7) - WRONG PART IN BOXES</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Orlando</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>KBMTEcpxxE29YvUx1XIW1WUAHWPC</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>ORLANDO - PO# 61462- INV T87878- PART # LC3Z7000JB- QTY  1- DATE 08.27.2024 - 9063054 Denied</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Orlando</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>NalqK5FqHUOuRfKZqz6LKmUAJqmL</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>ORLANDO - PO#  61607- INV U00965- PART#  J2GZ6006E- QTY  1- DATE 09.02.2024 - 9063720 Denied</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Orlando</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>NiJUAeMwYkWLqkR6TaCXZmUAK5TB</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>CHRYSLER OUTBOUND DAMAGE - 68515621AA - JERRY ULM CDJR - INV 3693836- CLAIM # ADL</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Orlando</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>_Bg1Cdqs3kyd-Db4KrbojWUAH4oz</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>ORLANDO - CHRYSLER SHORTAGE - PO 1301634 - 68393687AA - SHORT 1 - INV DATE 7.6.24 - CLAIM 172427 (C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Orlando</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>exo_QXUrgE6xetL_0_V56GUADnhg</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>CHRYSLER DAMAGE - PO# - 68447759AA - QTY 2  - INV 3263918 - WALLACE CJDR - CLAIM   002554</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Phoenix</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>-ACtth5XYk-YBOHBOfGOZWUAO5tw</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>LK4Z7000DA - #05534 - FRIENDLY FORD - S39-01356228 -</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Phoenix</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>3QKwH9g9nEqxR6PydFWu3WUAO_ey</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>CHRYSLER DAMAGE - PO# - 68346915AA - 2 EA - INV 3294016 LARRY H MILLER - CLAIM  986366 - 986367</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Phoenix</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>KFEY8ecMckiZEu47bBst9WUAIQlQ</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>CHRYSLER SHORTAGE - PO 0811804 - PART 68409357AA - SHORT 6 - INV DATE 3.30.24 - CLAIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Phoenix</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>LaT5IneeJUiF_Eo-LUadqGUADQlJ</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>PHOENIX - CHRYSLER SHORTAGE - PO 1310689- 68481771AA- SHORT 2 - INV DATE 02/28/2025 - CLAIM 858976 Denied</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Phoenix</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>MMs-KP85oUCl-fCMh8KjBWUABscA</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>PO# 160123 - S95396 - DA5Z7000ARM - 1 - 7.18.24</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Phoenix</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>NXuo-QVi6EWPjn55y6TQQWUAGaVZ</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>JC3Z7000JRM - PO 171840 - 05534 - FRIENDLY FORD - S39-01507418 - 3132854</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Phoenix</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>OF0FhSVwp0irDhcSFbIOJGUAI0fe</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>5C3Z7000MRM - PO 173688 - 20301 - SANDERSON REMAN - S39-01504194 - 3132797</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Phoenix</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Ut-bqiznV0iu9O8WV7CB5GUAD6Au</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>CHRYSLER SHORTAGE - PO 0820077 - P5160621AA - SHORT 1 - INV DATE 6.22.24 - CLAIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Phoenix</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>cYCjhp1n0kqVkIn-m0BaZ2UADQ3q</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>CHRYSLER PICK ERROR - SHORT 68498560AB - 1 - WRONG PART REC'D #68257658AE-QTY 2 - CLAIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Phoenix</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>wxszr3YEmUqTg2cKwZShqWUACHN2</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>JC3Z7000JRM - PO 171512 - 05534 - FRIENDLY FORD - IN01556054 - 3135920</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Phoenix</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>xTvHShtDtkeOn3Nlbq0-hmUAA8Kv</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>PICKING ERROR - PO# 0840817  - PART# 68237714BA - CLAIM 913712</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>